<commit_message>
fix: notebook ejecutable local y en Colab (orden gdf_zona_wgs + loop REFS); rasterio en requirements; gitignore de PNGs
</commit_message>
<xml_diff>
--- a/outputs/itt_ciudad_paraiso/ITT_Ciudad_Paraiso_Consolidado.xlsx
+++ b/outputs/itt_ciudad_paraiso/ITT_Ciudad_Paraiso_Consolidado.xlsx
@@ -11,7 +11,7 @@
     <sheet name="Seguridad" sheetId="2" state="visible" r:id="rId2"/>
     <sheet name="Movilidad" sheetId="3" state="visible" r:id="rId3"/>
     <sheet name="Cohesion_Social_DesSocial" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="Entorno_Urbano_proxy" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Entorno_Urbano_NDVI_arbol" sheetId="5" state="visible" r:id="rId5"/>
     <sheet name="Educacion_fuera_alcance" sheetId="6" state="visible" r:id="rId6"/>
     <sheet name="Desarrollo_Economico" sheetId="7" state="visible" r:id="rId7"/>
     <sheet name="Indicadores_Trimestrales" sheetId="8" state="visible" r:id="rId8"/>
@@ -508,13 +508,13 @@
         <v>59.81</v>
       </c>
       <c r="E2" t="n">
-        <v>70.2</v>
+        <v>51.35</v>
       </c>
       <c r="F2" t="n">
         <v>62.18</v>
       </c>
       <c r="G2" t="n">
-        <v>47.33</v>
+        <v>44.12</v>
       </c>
       <c r="H2" t="inlineStr">
         <is>
@@ -541,13 +541,13 @@
         <v>56</v>
       </c>
       <c r="E3" t="n">
-        <v>70.2</v>
+        <v>65.39</v>
       </c>
       <c r="F3" t="n">
         <v>67.94</v>
       </c>
       <c r="G3" t="n">
-        <v>56.32</v>
+        <v>55.5</v>
       </c>
       <c r="H3" t="inlineStr">
         <is>
@@ -574,13 +574,13 @@
         <v>31.38</v>
       </c>
       <c r="E4" t="n">
-        <v>70.2</v>
+        <v>65.2</v>
       </c>
       <c r="F4" t="n">
         <v>73.15000000000001</v>
       </c>
       <c r="G4" t="n">
-        <v>59.38</v>
+        <v>58.53</v>
       </c>
       <c r="H4" t="inlineStr">
         <is>
@@ -607,13 +607,13 @@
         <v>76.48</v>
       </c>
       <c r="E5" t="n">
-        <v>70.2</v>
+        <v>55.49</v>
       </c>
       <c r="F5" t="n">
         <v>73.15000000000001</v>
       </c>
       <c r="G5" t="n">
-        <v>83.86</v>
+        <v>81.36</v>
       </c>
       <c r="H5" t="inlineStr">
         <is>
@@ -1111,13 +1111,17 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D5"/>
+  <dimension ref="A1:H5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
-    <col width="17" customWidth="1" min="2" max="2"/>
-    <col width="40" customWidth="1" min="3" max="3"/>
-    <col width="40" customWidth="1" min="4" max="4"/>
+    <col width="8" customWidth="1" min="2" max="2"/>
+    <col width="10" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
+    <col width="16" customWidth="1" min="5" max="5"/>
+    <col width="17" customWidth="1" min="6" max="6"/>
+    <col width="40" customWidth="1" min="7" max="7"/>
+    <col width="40" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1128,15 +1132,35 @@
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
+          <t>ndvi</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>arbolado</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>score_ndvi</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>score_arbolado</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
           <t>score_entorno_u</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>fuente</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>nota</t>
         </is>
@@ -1147,16 +1171,28 @@
         <v>2023</v>
       </c>
       <c r="B2" t="n">
-        <v>70.2</v>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>Proxy por deficit habitacional (Comuna 3)</t>
-        </is>
-      </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>Proxy por deficit habitacional Comuna 3 — sin NDVI/arbolado propio de la zona</t>
+        <v>0.0948</v>
+      </c>
+      <c r="C2" t="n">
+        <v>303</v>
+      </c>
+      <c r="D2" t="n">
+        <v>35.9527</v>
+      </c>
+      <c r="E2" t="n">
+        <v>66.7401</v>
+      </c>
+      <c r="F2" t="n">
+        <v>51.3464</v>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>NDVI anual + censo arbóreo (datos propios de la zona)</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>NDVI medio anual (satelital) + censo arboreo vivo (corte unico). score_entorno_u = mean(score_ndvi, score_arbolado).</t>
         </is>
       </c>
     </row>
@@ -1165,16 +1201,28 @@
         <v>2024</v>
       </c>
       <c r="B3" t="n">
-        <v>70.2</v>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>Proxy por deficit habitacional (Comuna 3)</t>
-        </is>
-      </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>Proxy por deficit habitacional Comuna 3 — sin NDVI/arbolado propio de la zona</t>
+        <v>0.1102</v>
+      </c>
+      <c r="C3" t="n">
+        <v>303</v>
+      </c>
+      <c r="D3" t="n">
+        <v>64.04819999999999</v>
+      </c>
+      <c r="E3" t="n">
+        <v>66.7401</v>
+      </c>
+      <c r="F3" t="n">
+        <v>65.3942</v>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>NDVI anual + censo arbóreo (datos propios de la zona)</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>NDVI medio anual (satelital) + censo arboreo vivo (corte unico). score_entorno_u = mean(score_ndvi, score_arbolado).</t>
         </is>
       </c>
     </row>
@@ -1183,16 +1231,28 @@
         <v>2025</v>
       </c>
       <c r="B4" t="n">
-        <v>70.2</v>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>Proxy por deficit habitacional (Comuna 3)</t>
-        </is>
-      </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>Proxy por deficit habitacional Comuna 3 — sin NDVI/arbolado propio de la zona</t>
+        <v>0.11</v>
+      </c>
+      <c r="C4" t="n">
+        <v>303</v>
+      </c>
+      <c r="D4" t="n">
+        <v>63.6651</v>
+      </c>
+      <c r="E4" t="n">
+        <v>66.7401</v>
+      </c>
+      <c r="F4" t="n">
+        <v>65.2026</v>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>NDVI anual + censo arbóreo (datos propios de la zona)</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>NDVI medio anual (satelital) + censo arboreo vivo (corte unico). score_entorno_u = mean(score_ndvi, score_arbolado).</t>
         </is>
       </c>
     </row>
@@ -1201,16 +1261,28 @@
         <v>2026</v>
       </c>
       <c r="B5" t="n">
-        <v>70.2</v>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>Proxy por deficit habitacional (Comuna 3)</t>
-        </is>
-      </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>Proxy por deficit habitacional Comuna 3 — sin NDVI/arbolado propio de la zona</t>
+        <v>0.0993</v>
+      </c>
+      <c r="C5" t="n">
+        <v>303</v>
+      </c>
+      <c r="D5" t="n">
+        <v>44.2424</v>
+      </c>
+      <c r="E5" t="n">
+        <v>66.7401</v>
+      </c>
+      <c r="F5" t="n">
+        <v>55.4912</v>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>NDVI anual + censo arbóreo (datos propios de la zona)</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>NDVI medio anual (satelital) + censo arboreo vivo (corte unico). score_entorno_u = mean(score_ndvi, score_arbolado).</t>
         </is>
       </c>
     </row>
@@ -2118,7 +2190,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B7"/>
+  <dimension ref="A1:B8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -2209,6 +2281,18 @@
         </is>
       </c>
     </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Censo Arboreo</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Verificado 100% dentro del poligono via geopandas.sjoin (Celda 4B) al momento de esta corrida.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
feat(nb08): educacion completa (Camacho+Santa Librada: matricula/desercion/repitencia, fallback valores Colab), empleo DE desde registro 2025 (932 pers, 2026 vacio), colegios en Excel, sedes educativas en mapa; Excel regenerado
</commit_message>
<xml_diff>
--- a/outputs/itt_ciudad_paraiso/ITT_Ciudad_Paraiso_Consolidado.xlsx
+++ b/outputs/itt_ciudad_paraiso/ITT_Ciudad_Paraiso_Consolidado.xlsx
@@ -10,12 +10,12 @@
     <sheet name="ITT_Resumen" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="Seguridad" sheetId="2" state="visible" r:id="rId2"/>
     <sheet name="Movilidad" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Cohesion_Social_DesSocial" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="Entorno_Urbano_NDVI_arbol" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="Educacion_fuera_alcance" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="DesSocial_Cohesion_Educ" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Entorno_Urbano_NDVI_arb_viv" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Educacion" sheetId="6" state="visible" r:id="rId6"/>
     <sheet name="Desarrollo_Economico" sheetId="7" state="visible" r:id="rId7"/>
     <sheet name="Indicadores_Trimestrales" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet name="Auditoria_Spatial_Join" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet name="Auditoria_Fuentes" sheetId="9" state="visible" r:id="rId9"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -443,7 +443,7 @@
     <col width="17" customWidth="1" min="5" max="5"/>
     <col width="15" customWidth="1" min="6" max="6"/>
     <col width="7" customWidth="1" min="7" max="7"/>
-    <col width="25" customWidth="1" min="8" max="8"/>
+    <col width="16" customWidth="1" min="8" max="8"/>
     <col width="40" customWidth="1" min="9" max="9"/>
   </cols>
   <sheetData>
@@ -490,7 +490,7 @@
       </c>
       <c r="I1" s="1" t="inlineStr">
         <is>
-          <t>nota_estado</t>
+          <t>cobertura_2026</t>
         </is>
       </c>
     </row>
@@ -505,16 +505,16 @@
         <v>39.21</v>
       </c>
       <c r="D2" t="n">
-        <v>59.81</v>
+        <v>65.06</v>
       </c>
       <c r="E2" t="n">
-        <v>51.35</v>
+        <v>53.36</v>
       </c>
       <c r="F2" t="n">
-        <v>62.18</v>
+        <v>62.51</v>
       </c>
       <c r="G2" t="n">
-        <v>44.12</v>
+        <v>45.51</v>
       </c>
       <c r="H2" t="inlineStr">
         <is>
@@ -523,7 +523,7 @@
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>Real</t>
+          <t>Año completo</t>
         </is>
       </c>
     </row>
@@ -538,16 +538,16 @@
         <v>35.71</v>
       </c>
       <c r="D3" t="n">
-        <v>56</v>
+        <v>52.86</v>
       </c>
       <c r="E3" t="n">
+        <v>62.73</v>
+      </c>
+      <c r="F3" t="n">
         <v>65.39</v>
       </c>
-      <c r="F3" t="n">
-        <v>67.94</v>
-      </c>
       <c r="G3" t="n">
-        <v>55.5</v>
+        <v>54.07</v>
       </c>
       <c r="H3" t="inlineStr">
         <is>
@@ -556,7 +556,7 @@
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>Real</t>
+          <t>Año completo</t>
         </is>
       </c>
     </row>
@@ -571,16 +571,16 @@
         <v>71.19</v>
       </c>
       <c r="D4" t="n">
-        <v>31.38</v>
+        <v>32.1</v>
       </c>
       <c r="E4" t="n">
-        <v>65.2</v>
+        <v>62.6</v>
       </c>
       <c r="F4" t="n">
-        <v>73.15000000000001</v>
+        <v>68.56</v>
       </c>
       <c r="G4" t="n">
-        <v>58.53</v>
+        <v>57.54</v>
       </c>
       <c r="H4" t="inlineStr">
         <is>
@@ -589,7 +589,7 @@
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>Real</t>
+          <t>Año completo</t>
         </is>
       </c>
     </row>
@@ -598,31 +598,31 @@
         <v>2026</v>
       </c>
       <c r="B5" t="n">
-        <v>95</v>
+        <v>88.12</v>
       </c>
       <c r="C5" t="n">
         <v>94.44</v>
       </c>
       <c r="D5" t="n">
-        <v>76.48</v>
+        <v>16.9</v>
       </c>
       <c r="E5" t="n">
-        <v>55.49</v>
+        <v>56.13</v>
       </c>
       <c r="F5" t="n">
-        <v>73.15000000000001</v>
+        <v>61.17</v>
       </c>
       <c r="G5" t="n">
-        <v>81.36</v>
+        <v>66.5</v>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>Parcial (no comparable)</t>
+          <t>Transformacion</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>Parcial (no comparable) | cobertura incompleta en todas las fuentes | DesEco referencial 2025</t>
+          <t>DATIC Q1-Q3 | siniestros Q1-Q2 | resto año en curso</t>
         </is>
       </c>
     </row>
@@ -745,19 +745,19 @@
         <v>2026</v>
       </c>
       <c r="B5" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="C5" t="n">
-        <v>44</v>
+        <v>89</v>
       </c>
       <c r="D5" t="n">
-        <v>90</v>
+        <v>80</v>
       </c>
       <c r="E5" t="n">
-        <v>100</v>
+        <v>96.25</v>
       </c>
       <c r="F5" t="n">
-        <v>95</v>
+        <v>88.12</v>
       </c>
     </row>
   </sheetData>
@@ -941,7 +941,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H5"/>
+  <dimension ref="A1:J5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -951,7 +951,9 @@
     <col width="11" customWidth="1" min="5" max="5"/>
     <col width="13" customWidth="1" min="6" max="6"/>
     <col width="11" customWidth="1" min="7" max="7"/>
-    <col width="26" customWidth="1" min="8" max="8"/>
+    <col width="17" customWidth="1" min="8" max="8"/>
+    <col width="17" customWidth="1" min="9" max="9"/>
+    <col width="17" customWidth="1" min="10" max="10"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -992,7 +994,17 @@
       </c>
       <c r="H1" s="1" t="inlineStr">
         <is>
-          <t>score_cohesion_DesSocial</t>
+          <t>score_matricula</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>score_desercion</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>score_DesSocial</t>
         </is>
       </c>
     </row>
@@ -1019,7 +1031,13 @@
         <v>60</v>
       </c>
       <c r="H2" t="n">
-        <v>59.81</v>
+        <v>100</v>
+      </c>
+      <c r="I2" t="n">
+        <v>45.87</v>
+      </c>
+      <c r="J2" t="n">
+        <v>65.06</v>
       </c>
     </row>
     <row r="3">
@@ -1045,7 +1063,13 @@
         <v>87.14</v>
       </c>
       <c r="H3" t="n">
-        <v>56</v>
+        <v>37.69</v>
+      </c>
+      <c r="I3" t="n">
+        <v>58.6</v>
+      </c>
+      <c r="J3" t="n">
+        <v>52.86</v>
       </c>
     </row>
     <row r="4">
@@ -1071,7 +1095,13 @@
         <v>20.71</v>
       </c>
       <c r="H4" t="n">
-        <v>31.38</v>
+        <v>0</v>
+      </c>
+      <c r="I4" t="n">
+        <v>66.33</v>
+      </c>
+      <c r="J4" t="n">
+        <v>32.1</v>
       </c>
     </row>
     <row r="5">
@@ -1079,25 +1109,27 @@
         <v>2026</v>
       </c>
       <c r="B5" t="n">
-        <v>12</v>
+        <v>17</v>
       </c>
       <c r="C5" t="n">
-        <v>157</v>
+        <v>547</v>
       </c>
       <c r="D5" t="n">
-        <v>57</v>
+        <v>135</v>
       </c>
       <c r="E5" t="n">
-        <v>65</v>
+        <v>40</v>
       </c>
       <c r="F5" t="n">
-        <v>98</v>
+        <v>0</v>
       </c>
       <c r="G5" t="n">
-        <v>66.43000000000001</v>
-      </c>
-      <c r="H5" t="n">
-        <v>76.48</v>
+        <v>10.71</v>
+      </c>
+      <c r="H5" t="inlineStr"/>
+      <c r="I5" t="inlineStr"/>
+      <c r="J5" t="n">
+        <v>16.9</v>
       </c>
     </row>
   </sheetData>
@@ -1111,7 +1143,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H5"/>
+  <dimension ref="A1:I5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -1119,9 +1151,10 @@
     <col width="10" customWidth="1" min="3" max="3"/>
     <col width="12" customWidth="1" min="4" max="4"/>
     <col width="16" customWidth="1" min="5" max="5"/>
-    <col width="17" customWidth="1" min="6" max="6"/>
-    <col width="40" customWidth="1" min="7" max="7"/>
+    <col width="21" customWidth="1" min="6" max="6"/>
+    <col width="17" customWidth="1" min="7" max="7"/>
     <col width="40" customWidth="1" min="8" max="8"/>
+    <col width="40" customWidth="1" min="9" max="9"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1152,15 +1185,20 @@
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
+          <t>score_habitabilidad</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
           <t>score_entorno_u</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>fuente</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>nota</t>
         </is>
@@ -1183,16 +1221,19 @@
         <v>66.7401</v>
       </c>
       <c r="F2" t="n">
-        <v>51.3464</v>
-      </c>
-      <c r="G2" t="inlineStr">
+        <v>57.4</v>
+      </c>
+      <c r="G2" t="n">
+        <v>53.3643</v>
+      </c>
+      <c r="H2" t="inlineStr">
         <is>
           <t>NDVI anual + censo arbóreo (datos propios de la zona)</t>
         </is>
       </c>
-      <c r="H2" t="inlineStr">
-        <is>
-          <t>NDVI medio anual (satelital) + censo arboreo vivo (corte unico). score_entorno_u = mean(score_ndvi, score_arbolado).</t>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>NDVI anual satelital + censo arbóreo + habitabilidad (1 - déficit habitacional 2024). Vivienda es corte único estructural 2024 (constante en la serie).</t>
         </is>
       </c>
     </row>
@@ -1213,16 +1254,19 @@
         <v>66.7401</v>
       </c>
       <c r="F3" t="n">
-        <v>65.3942</v>
-      </c>
-      <c r="G3" t="inlineStr">
+        <v>57.4</v>
+      </c>
+      <c r="G3" t="n">
+        <v>62.7294</v>
+      </c>
+      <c r="H3" t="inlineStr">
         <is>
           <t>NDVI anual + censo arbóreo (datos propios de la zona)</t>
         </is>
       </c>
-      <c r="H3" t="inlineStr">
-        <is>
-          <t>NDVI medio anual (satelital) + censo arboreo vivo (corte unico). score_entorno_u = mean(score_ndvi, score_arbolado).</t>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>NDVI anual satelital + censo arbóreo + habitabilidad (1 - déficit habitacional 2024). Vivienda es corte único estructural 2024 (constante en la serie).</t>
         </is>
       </c>
     </row>
@@ -1243,16 +1287,19 @@
         <v>66.7401</v>
       </c>
       <c r="F4" t="n">
-        <v>65.2026</v>
-      </c>
-      <c r="G4" t="inlineStr">
+        <v>57.4</v>
+      </c>
+      <c r="G4" t="n">
+        <v>62.6017</v>
+      </c>
+      <c r="H4" t="inlineStr">
         <is>
           <t>NDVI anual + censo arbóreo (datos propios de la zona)</t>
         </is>
       </c>
-      <c r="H4" t="inlineStr">
-        <is>
-          <t>NDVI medio anual (satelital) + censo arboreo vivo (corte unico). score_entorno_u = mean(score_ndvi, score_arbolado).</t>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>NDVI anual satelital + censo arbóreo + habitabilidad (1 - déficit habitacional 2024). Vivienda es corte único estructural 2024 (constante en la serie).</t>
         </is>
       </c>
     </row>
@@ -1273,16 +1320,19 @@
         <v>66.7401</v>
       </c>
       <c r="F5" t="n">
-        <v>55.4912</v>
-      </c>
-      <c r="G5" t="inlineStr">
+        <v>57.4</v>
+      </c>
+      <c r="G5" t="n">
+        <v>56.1275</v>
+      </c>
+      <c r="H5" t="inlineStr">
         <is>
           <t>NDVI anual + censo arbóreo (datos propios de la zona)</t>
         </is>
       </c>
-      <c r="H5" t="inlineStr">
-        <is>
-          <t>NDVI medio anual (satelital) + censo arboreo vivo (corte unico). score_entorno_u = mean(score_ndvi, score_arbolado).</t>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>NDVI anual satelital + censo arbóreo + habitabilidad (1 - déficit habitacional 2024). Vivienda es corte único estructural 2024 (constante en la serie).</t>
         </is>
       </c>
     </row>
@@ -1297,37 +1347,187 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A4"/>
+  <dimension ref="A1:K4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="40" customWidth="1" min="1" max="1"/>
+    <col width="6" customWidth="1" min="1" max="1"/>
+    <col width="11" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
+    <col width="16" customWidth="1" min="5" max="5"/>
+    <col width="17" customWidth="1" min="6" max="6"/>
+    <col width="17" customWidth="1" min="7" max="7"/>
+    <col width="18" customWidth="1" min="8" max="8"/>
+    <col width="16" customWidth="1" min="9" max="9"/>
+    <col width="17" customWidth="1" min="10" max="10"/>
+    <col width="40" customWidth="1" min="11" max="11"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>nota</t>
+          <t>año</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>matricula</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>desertores</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>repitentes</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>tasa_desercion</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>tasa_repitencia</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>score_desercion</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>score_repitencia</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>score_educ_des</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>score_matricula</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>colegios</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>Educacion y Desarrollo NO se calcula en este repositorio.</t>
+      <c r="A2" t="n">
+        <v>2023</v>
+      </c>
+      <c r="B2" t="n">
+        <v>3891</v>
+      </c>
+      <c r="C2" t="n">
+        <v>316</v>
+      </c>
+      <c r="D2" t="n">
+        <v>365</v>
+      </c>
+      <c r="E2" t="n">
+        <v>8.119999999999999</v>
+      </c>
+      <c r="F2" t="n">
+        <v>9.380000000000001</v>
+      </c>
+      <c r="G2" t="n">
+        <v>45.87</v>
+      </c>
+      <c r="H2" t="n">
+        <v>53.1</v>
+      </c>
+      <c r="I2" t="n">
+        <v>49.5</v>
+      </c>
+      <c r="J2" t="n">
+        <v>100</v>
+      </c>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>IE Antonio José Camacho (176001001753) + IE Santa Librada (176001001818)</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>Se gestiona en otro repositorio (indicacion del usuario, 2026-10-04).</t>
+      <c r="A3" t="n">
+        <v>2024</v>
+      </c>
+      <c r="B3" t="n">
+        <v>3529</v>
+      </c>
+      <c r="C3" t="n">
+        <v>219</v>
+      </c>
+      <c r="D3" t="n">
+        <v>367</v>
+      </c>
+      <c r="E3" t="n">
+        <v>6.21</v>
+      </c>
+      <c r="F3" t="n">
+        <v>10.4</v>
+      </c>
+      <c r="G3" t="n">
+        <v>58.6</v>
+      </c>
+      <c r="H3" t="n">
+        <v>48</v>
+      </c>
+      <c r="I3" t="n">
+        <v>53.3</v>
+      </c>
+      <c r="J3" t="n">
+        <v>37.69</v>
+      </c>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>IE Antonio José Camacho (176001001753) + IE Santa Librada (176001001818)</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>La dimension DesSocial de este notebook usa unicamente VIF + Rinas + SPA.</t>
+      <c r="A4" t="n">
+        <v>2025</v>
+      </c>
+      <c r="B4" t="n">
+        <v>3310</v>
+      </c>
+      <c r="C4" t="n">
+        <v>167</v>
+      </c>
+      <c r="D4" t="n">
+        <v>302</v>
+      </c>
+      <c r="E4" t="n">
+        <v>5.05</v>
+      </c>
+      <c r="F4" t="n">
+        <v>9.119999999999999</v>
+      </c>
+      <c r="G4" t="n">
+        <v>66.33</v>
+      </c>
+      <c r="H4" t="n">
+        <v>54.4</v>
+      </c>
+      <c r="I4" t="n">
+        <v>60.4</v>
+      </c>
+      <c r="J4" t="n">
+        <v>0</v>
+      </c>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>IE Antonio José Camacho (176001001753) + IE Santa Librada (176001001818)</t>
         </is>
       </c>
     </row>
@@ -1342,19 +1542,22 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J5"/>
+  <dimension ref="A1:M5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
     <col width="40" customWidth="1" min="2" max="2"/>
     <col width="26" customWidth="1" min="3" max="3"/>
-    <col width="21" customWidth="1" min="4" max="4"/>
-    <col width="24" customWidth="1" min="5" max="5"/>
-    <col width="16" customWidth="1" min="6" max="6"/>
-    <col width="24" customWidth="1" min="7" max="7"/>
-    <col width="21" customWidth="1" min="8" max="8"/>
-    <col width="16" customWidth="1" min="9" max="9"/>
-    <col width="15" customWidth="1" min="10" max="10"/>
+    <col width="24" customWidth="1" min="4" max="4"/>
+    <col width="16" customWidth="1" min="5" max="5"/>
+    <col width="17" customWidth="1" min="6" max="6"/>
+    <col width="16" customWidth="1" min="7" max="7"/>
+    <col width="14" customWidth="1" min="8" max="8"/>
+    <col width="24" customWidth="1" min="9" max="9"/>
+    <col width="16" customWidth="1" min="10" max="10"/>
+    <col width="20" customWidth="1" min="11" max="11"/>
+    <col width="14" customWidth="1" min="12" max="12"/>
+    <col width="15" customWidth="1" min="13" max="13"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1375,35 +1578,50 @@
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>empleabilidad_total</t>
+          <t>ingresos_operacionales</t>
         </is>
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
-          <t>ingresos_operacionales</t>
+          <t>activo_total</t>
         </is>
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
+          <t>empleo_personas</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
           <t>ingresos_log1p</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>activo_log1p</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>score_establecimientos</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
-        <is>
-          <t>score_empleabilidad</t>
-        </is>
-      </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>score_ingresos</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>score_activo_total</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>score_empleo</t>
+        </is>
+      </c>
+      <c r="M1" s="1" t="inlineStr">
         <is>
           <t>score_des_eco</t>
         </is>
@@ -1415,32 +1633,41 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Proxy retrospectivo (stock acumulado hasta ese año)</t>
+          <t>Real (stock activo, fuente consolidada)</t>
         </is>
       </c>
       <c r="C2" t="n">
-        <v>259</v>
+        <v>236</v>
       </c>
       <c r="D2" t="n">
-        <v>868</v>
+        <v>374307227177</v>
       </c>
       <c r="E2" t="n">
-        <v>600156325931</v>
+        <v>527574501397</v>
       </c>
       <c r="F2" t="n">
-        <v>27.12</v>
+        <v>932</v>
       </c>
       <c r="G2" t="n">
-        <v>45.43</v>
+        <v>26.65</v>
       </c>
       <c r="H2" t="n">
-        <v>63.11</v>
+        <v>26.99</v>
       </c>
       <c r="I2" t="n">
-        <v>78.01000000000001</v>
+        <v>63.27</v>
       </c>
       <c r="J2" t="n">
-        <v>62.18</v>
+        <v>49.95</v>
+      </c>
+      <c r="K2" t="n">
+        <v>49.87</v>
+      </c>
+      <c r="L2" t="n">
+        <v>86.95999999999999</v>
+      </c>
+      <c r="M2" t="n">
+        <v>62.51</v>
       </c>
     </row>
     <row r="3">
@@ -1449,32 +1676,41 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Proxy retrospectivo (stock acumulado hasta ese año)</t>
+          <t>Real (stock activo, fuente consolidada)</t>
         </is>
       </c>
       <c r="C3" t="n">
-        <v>301</v>
+        <v>278</v>
       </c>
       <c r="D3" t="n">
-        <v>915</v>
+        <v>374657166989</v>
       </c>
       <c r="E3" t="n">
-        <v>601623288743</v>
+        <v>528536097126</v>
       </c>
       <c r="F3" t="n">
-        <v>27.12</v>
+        <v>932</v>
       </c>
       <c r="G3" t="n">
-        <v>57.43</v>
+        <v>26.65</v>
       </c>
       <c r="H3" t="n">
-        <v>68.33</v>
+        <v>26.99</v>
       </c>
       <c r="I3" t="n">
-        <v>78.06999999999999</v>
+        <v>74.53</v>
       </c>
       <c r="J3" t="n">
-        <v>67.94</v>
+        <v>50.04</v>
+      </c>
+      <c r="K3" t="n">
+        <v>50.04</v>
+      </c>
+      <c r="L3" t="n">
+        <v>86.95999999999999</v>
+      </c>
+      <c r="M3" t="n">
+        <v>65.39</v>
       </c>
     </row>
     <row r="4">
@@ -1483,32 +1719,41 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Real</t>
+          <t>Real (stock activo, fuente consolidada)</t>
         </is>
       </c>
       <c r="C4" t="n">
-        <v>349</v>
+        <v>325</v>
       </c>
       <c r="D4" t="n">
+        <v>374690467989</v>
+      </c>
+      <c r="E4" t="n">
+        <v>529034175386</v>
+      </c>
+      <c r="F4" t="n">
         <v>932</v>
       </c>
-      <c r="E4" t="n">
-        <v>601634389743</v>
-      </c>
-      <c r="F4" t="n">
-        <v>27.12</v>
-      </c>
       <c r="G4" t="n">
-        <v>71.14</v>
+        <v>26.65</v>
       </c>
       <c r="H4" t="n">
-        <v>70.22</v>
+        <v>26.99</v>
       </c>
       <c r="I4" t="n">
-        <v>78.06999999999999</v>
+        <v>87.13</v>
       </c>
       <c r="J4" t="n">
-        <v>73.15000000000001</v>
+        <v>50.05</v>
+      </c>
+      <c r="K4" t="n">
+        <v>50.13</v>
+      </c>
+      <c r="L4" t="n">
+        <v>86.95999999999999</v>
+      </c>
+      <c r="M4" t="n">
+        <v>68.56</v>
       </c>
     </row>
     <row r="5">
@@ -1517,32 +1762,37 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Proxy referencial = 2025 (sin corte 2026 disponible)</t>
+          <t>Real (stock activo, fuente consolidada)</t>
         </is>
       </c>
       <c r="C5" t="n">
-        <v>349</v>
+        <v>311</v>
       </c>
       <c r="D5" t="n">
-        <v>932</v>
+        <v>374685467989</v>
       </c>
       <c r="E5" t="n">
-        <v>601634389743</v>
-      </c>
-      <c r="F5" t="n">
-        <v>27.12</v>
-      </c>
+        <v>528743475386</v>
+      </c>
+      <c r="F5" t="inlineStr"/>
       <c r="G5" t="n">
-        <v>71.14</v>
+        <v>26.65</v>
       </c>
       <c r="H5" t="n">
-        <v>70.22</v>
+        <v>26.99</v>
       </c>
       <c r="I5" t="n">
-        <v>78.06999999999999</v>
+        <v>83.38</v>
       </c>
       <c r="J5" t="n">
-        <v>73.15000000000001</v>
+        <v>50.05</v>
+      </c>
+      <c r="K5" t="n">
+        <v>50.07</v>
+      </c>
+      <c r="L5" t="inlineStr"/>
+      <c r="M5" t="n">
+        <v>61.17</v>
       </c>
     </row>
   </sheetData>
@@ -2117,8 +2367,12 @@
       <c r="B15" t="n">
         <v>2</v>
       </c>
-      <c r="C15" t="inlineStr"/>
-      <c r="D15" t="inlineStr"/>
+      <c r="C15" t="n">
+        <v>0</v>
+      </c>
+      <c r="D15" t="n">
+        <v>23</v>
+      </c>
       <c r="E15" t="n">
         <v>1</v>
       </c>
@@ -2128,9 +2382,15 @@
       <c r="G15" t="n">
         <v>0</v>
       </c>
-      <c r="H15" t="inlineStr"/>
-      <c r="I15" t="inlineStr"/>
-      <c r="J15" t="inlineStr"/>
+      <c r="H15" t="n">
+        <v>2</v>
+      </c>
+      <c r="I15" t="n">
+        <v>217</v>
+      </c>
+      <c r="J15" t="n">
+        <v>57</v>
+      </c>
       <c r="K15" t="inlineStr">
         <is>
           <t>2026-Q2</t>
@@ -2144,14 +2404,24 @@
       <c r="B16" t="n">
         <v>3</v>
       </c>
-      <c r="C16" t="inlineStr"/>
-      <c r="D16" t="inlineStr"/>
+      <c r="C16" t="n">
+        <v>2</v>
+      </c>
+      <c r="D16" t="n">
+        <v>22</v>
+      </c>
       <c r="E16" t="inlineStr"/>
       <c r="F16" t="inlineStr"/>
       <c r="G16" t="inlineStr"/>
-      <c r="H16" t="inlineStr"/>
-      <c r="I16" t="inlineStr"/>
-      <c r="J16" t="inlineStr"/>
+      <c r="H16" t="n">
+        <v>3</v>
+      </c>
+      <c r="I16" t="n">
+        <v>173</v>
+      </c>
+      <c r="J16" t="n">
+        <v>21</v>
+      </c>
       <c r="K16" t="inlineStr">
         <is>
           <t>2026-Q3</t>
@@ -2190,10 +2460,10 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B8"/>
+  <dimension ref="A1:B10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="20" customWidth="1" min="1" max="1"/>
+    <col width="34" customWidth="1" min="1" max="1"/>
     <col width="40" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
@@ -2217,7 +2487,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Verificado 100% dentro del poligono via geopandas.sjoin (Celda 4B) al momento de esta corrida.</t>
+          <t>Línea base por verificación espacial (Celda 4B); extensiones 2026 por spatial join al polígono.</t>
         </is>
       </c>
     </row>
@@ -2229,7 +2499,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Verificado 100% dentro del poligono via geopandas.sjoin (Celda 4B) al momento de esta corrida.</t>
+          <t>Línea base por verificación espacial (Celda 4B); extensiones 2026 por spatial join al polígono.</t>
         </is>
       </c>
     </row>
@@ -2241,7 +2511,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Verificado 100% dentro del poligono via geopandas.sjoin (Celda 4B) al momento de esta corrida.</t>
+          <t>Línea base por verificación espacial (Celda 4B); extensiones 2026 por spatial join al polígono.</t>
         </is>
       </c>
     </row>
@@ -2253,7 +2523,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Verificado 100% dentro del poligono via geopandas.sjoin (Celda 4B) al momento de esta corrida.</t>
+          <t>Línea base por verificación espacial (Celda 4B); extensiones 2026 por spatial join al polígono.</t>
         </is>
       </c>
     </row>
@@ -2265,19 +2535,19 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Verificado 100% dentro del poligono via geopandas.sjoin (Celda 4B) al momento de esta corrida.</t>
+          <t>Línea base por verificación espacial (Celda 4B); extensiones 2026 por spatial join al polígono.</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Registro Mercantil</t>
+          <t>Registro Mercantil (consolidado)</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Verificado 100% dentro del poligono via geopandas.sjoin (Celda 4B) al momento de esta corrida.</t>
+          <t>Línea base por verificación espacial (Celda 4B); extensiones 2026 por spatial join al polígono.</t>
         </is>
       </c>
     </row>
@@ -2289,7 +2559,31 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Verificado 100% dentro del poligono via geopandas.sjoin (Celda 4B) al momento de esta corrida.</t>
+          <t>Línea base por verificación espacial (Celda 4B); extensiones 2026 por spatial join al polígono.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Déficit Habitacional 2024</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Línea base por verificación espacial (Celda 4B); extensiones 2026 por spatial join al polígono.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Educación SIMPADE</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Línea base por verificación espacial (Celda 4B); extensiones 2026 por spatial join al polígono.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat(nb08): educacion 2026 (corte marzo SIMAT: matricula 3276, repitentes 317; desercion vacia sin SIMPADE 2026); ignorar carpeta Educacion_2026 (archivos 40MB); Excel regenerado con educacion 2023-2026
</commit_message>
<xml_diff>
--- a/outputs/itt_ciudad_paraiso/ITT_Ciudad_Paraiso_Consolidado.xlsx
+++ b/outputs/itt_ciudad_paraiso/ITT_Ciudad_Paraiso_Consolidado.xlsx
@@ -538,7 +538,7 @@
         <v>35.71</v>
       </c>
       <c r="D3" t="n">
-        <v>52.86</v>
+        <v>53.55</v>
       </c>
       <c r="E3" t="n">
         <v>62.73</v>
@@ -547,7 +547,7 @@
         <v>64.98</v>
       </c>
       <c r="G3" t="n">
-        <v>54</v>
+        <v>54.14</v>
       </c>
       <c r="H3" t="inlineStr">
         <is>
@@ -571,7 +571,7 @@
         <v>71.19</v>
       </c>
       <c r="D4" t="n">
-        <v>32.1</v>
+        <v>33.2</v>
       </c>
       <c r="E4" t="n">
         <v>62.6</v>
@@ -580,7 +580,7 @@
         <v>68.56</v>
       </c>
       <c r="G4" t="n">
-        <v>57.54</v>
+        <v>57.75</v>
       </c>
       <c r="H4" t="inlineStr">
         <is>
@@ -604,7 +604,7 @@
         <v>94.44</v>
       </c>
       <c r="D5" t="n">
-        <v>16.9</v>
+        <v>12.68</v>
       </c>
       <c r="E5" t="n">
         <v>56.13</v>
@@ -613,7 +613,7 @@
         <v>67.3</v>
       </c>
       <c r="G5" t="n">
-        <v>67.42</v>
+        <v>66.62</v>
       </c>
       <c r="H5" t="inlineStr">
         <is>
@@ -1063,13 +1063,13 @@
         <v>87.14</v>
       </c>
       <c r="H3" t="n">
-        <v>37.69</v>
+        <v>41.14</v>
       </c>
       <c r="I3" t="n">
         <v>58.6</v>
       </c>
       <c r="J3" t="n">
-        <v>52.86</v>
+        <v>53.55</v>
       </c>
     </row>
     <row r="4">
@@ -1095,13 +1095,13 @@
         <v>20.71</v>
       </c>
       <c r="H4" t="n">
-        <v>0</v>
+        <v>5.53</v>
       </c>
       <c r="I4" t="n">
         <v>66.33</v>
       </c>
       <c r="J4" t="n">
-        <v>32.1</v>
+        <v>33.2</v>
       </c>
     </row>
     <row r="5">
@@ -1126,10 +1126,12 @@
       <c r="G5" t="n">
         <v>10.71</v>
       </c>
-      <c r="H5" t="inlineStr"/>
+      <c r="H5" t="n">
+        <v>0</v>
+      </c>
       <c r="I5" t="inlineStr"/>
       <c r="J5" t="n">
-        <v>16.9</v>
+        <v>12.68</v>
       </c>
     </row>
   </sheetData>
@@ -1347,7 +1349,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K4"/>
+  <dimension ref="A1:K5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -1486,7 +1488,7 @@
         <v>53.3</v>
       </c>
       <c r="J3" t="n">
-        <v>37.69</v>
+        <v>41.14</v>
       </c>
       <c r="K3" t="inlineStr">
         <is>
@@ -1523,9 +1525,40 @@
         <v>60.4</v>
       </c>
       <c r="J4" t="n">
+        <v>5.53</v>
+      </c>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>IE Antonio José Camacho (176001001753) + IE Santa Librada (176001001818)</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="n">
+        <v>2026</v>
+      </c>
+      <c r="B5" t="n">
+        <v>3276</v>
+      </c>
+      <c r="C5" t="inlineStr"/>
+      <c r="D5" t="n">
+        <v>317</v>
+      </c>
+      <c r="E5" t="inlineStr"/>
+      <c r="F5" t="n">
+        <v>9.68</v>
+      </c>
+      <c r="G5" t="inlineStr"/>
+      <c r="H5" t="n">
+        <v>51.6</v>
+      </c>
+      <c r="I5" t="n">
+        <v>51.6</v>
+      </c>
+      <c r="J5" t="n">
         <v>0</v>
       </c>
-      <c r="K4" t="inlineStr">
+      <c r="K5" t="inlineStr">
         <is>
           <t>IE Antonio José Camacho (176001001753) + IE Santa Librada (176001001818)</t>
         </is>

</xml_diff>

<commit_message>
feat(nb08): hoja Vivienda_SecVivienda en Excel — deficit habitacional por los 15 barrios de Ciudad Paraiso (Comuna 3) con tasas, totales y fuente Secretaria de Vivienda
</commit_message>
<xml_diff>
--- a/outputs/itt_ciudad_paraiso/ITT_Ciudad_Paraiso_Consolidado.xlsx
+++ b/outputs/itt_ciudad_paraiso/ITT_Ciudad_Paraiso_Consolidado.xlsx
@@ -12,10 +12,11 @@
     <sheet name="Movilidad" sheetId="3" state="visible" r:id="rId3"/>
     <sheet name="DesSocial_Cohesion_Educ" sheetId="4" state="visible" r:id="rId4"/>
     <sheet name="Entorno_Urbano_NDVI_arb_viv" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="Educacion" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="Desarrollo_Economico" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet name="Indicadores_Trimestrales" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet name="Auditoria_Fuentes" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet name="Vivienda_SecVivienda" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="Educacion" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="Desarrollo_Economico" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="Indicadores_Trimestrales" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet name="Auditoria_Fuentes" sheetId="10" state="visible" r:id="rId10"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -631,6 +632,144 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:B10"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="34" customWidth="1" min="1" max="1"/>
+    <col width="40" customWidth="1" min="2" max="2"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>fuente</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>nota</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Homicidios</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Línea base por verificación espacial (Celda 4B); extensiones 2026 por spatial join al polígono.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Hurtos</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Línea base por verificación espacial (Celda 4B); extensiones 2026 por spatial join al polígono.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Comparendos</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Línea base por verificación espacial (Celda 4B); extensiones 2026 por spatial join al polígono.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>VIF</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Línea base por verificación espacial (Celda 4B); extensiones 2026 por spatial join al polígono.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Siniestros</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Línea base por verificación espacial (Celda 4B); extensiones 2026 por spatial join al polígono.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Registro Mercantil (consolidado)</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Línea base por verificación espacial (Celda 4B); extensiones 2026 por spatial join al polígono.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Censo Arboreo</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Línea base por verificación espacial (Celda 4B); extensiones 2026 por spatial join al polígono.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Déficit Habitacional 2024</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Línea base por verificación espacial (Celda 4B); extensiones 2026 por spatial join al polígono.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Educación SIMPADE</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Línea base por verificación espacial (Celda 4B); extensiones 2026 por spatial join al polígono.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
@@ -1349,6 +1488,552 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:H17"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="33" customWidth="1" min="1" max="1"/>
+    <col width="15" customWidth="1" min="2" max="2"/>
+    <col width="22" customWidth="1" min="3" max="3"/>
+    <col width="22" customWidth="1" min="4" max="4"/>
+    <col width="21" customWidth="1" min="5" max="5"/>
+    <col width="16" customWidth="1" min="6" max="6"/>
+    <col width="21" customWidth="1" min="7" max="7"/>
+    <col width="40" customWidth="1" min="8" max="8"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>barrio</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>total_hogares</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>deficit_habitacional</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>deficit_cuantitativo</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>deficit_cualitativo</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>tasa_deficit_%</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>habitabilidad_score</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>fuente</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>El Nacional</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
+        <v>470</v>
+      </c>
+      <c r="C2" t="n">
+        <v>198</v>
+      </c>
+      <c r="D2" t="n">
+        <v>17</v>
+      </c>
+      <c r="E2" t="n">
+        <v>181</v>
+      </c>
+      <c r="F2" t="n">
+        <v>42.1</v>
+      </c>
+      <c r="G2" t="n">
+        <v>57.4</v>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>Secretaría de Vivienda - Déficit Habitacional por barrios 2024 (SISBÉN). Corte único estructural.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>El Peñón</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>12</v>
+      </c>
+      <c r="C3" t="n">
+        <v>6</v>
+      </c>
+      <c r="D3" t="n">
+        <v>0</v>
+      </c>
+      <c r="E3" t="n">
+        <v>6</v>
+      </c>
+      <c r="F3" t="n">
+        <v>50</v>
+      </c>
+      <c r="G3" t="n">
+        <v>57.4</v>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>Secretaría de Vivienda - Déficit Habitacional por barrios 2024 (SISBÉN). Corte único estructural.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>San Antonio</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>216</v>
+      </c>
+      <c r="C4" t="n">
+        <v>94</v>
+      </c>
+      <c r="D4" t="n">
+        <v>6</v>
+      </c>
+      <c r="E4" t="n">
+        <v>88</v>
+      </c>
+      <c r="F4" t="n">
+        <v>43.5</v>
+      </c>
+      <c r="G4" t="n">
+        <v>57.4</v>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>Secretaría de Vivienda - Déficit Habitacional por barrios 2024 (SISBÉN). Corte único estructural.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>San Cayetano</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>754</v>
+      </c>
+      <c r="C5" t="n">
+        <v>240</v>
+      </c>
+      <c r="D5" t="n">
+        <v>12</v>
+      </c>
+      <c r="E5" t="n">
+        <v>228</v>
+      </c>
+      <c r="F5" t="n">
+        <v>31.8</v>
+      </c>
+      <c r="G5" t="n">
+        <v>57.4</v>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>Secretaría de Vivienda - Déficit Habitacional por barrios 2024 (SISBÉN). Corte único estructural.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Los Libertadores</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>629</v>
+      </c>
+      <c r="C6" t="n">
+        <v>218</v>
+      </c>
+      <c r="D6" t="n">
+        <v>15</v>
+      </c>
+      <c r="E6" t="n">
+        <v>203</v>
+      </c>
+      <c r="F6" t="n">
+        <v>34.7</v>
+      </c>
+      <c r="G6" t="n">
+        <v>57.4</v>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>Secretaría de Vivienda - Déficit Habitacional por barrios 2024 (SISBÉN). Corte único estructural.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>San Juan Bosco</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>1120</v>
+      </c>
+      <c r="C7" t="n">
+        <v>558</v>
+      </c>
+      <c r="D7" t="n">
+        <v>158</v>
+      </c>
+      <c r="E7" t="n">
+        <v>400</v>
+      </c>
+      <c r="F7" t="n">
+        <v>49.8</v>
+      </c>
+      <c r="G7" t="n">
+        <v>57.4</v>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>Secretaría de Vivienda - Déficit Habitacional por barrios 2024 (SISBÉN). Corte único estructural.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Santa Rosa</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>412</v>
+      </c>
+      <c r="C8" t="n">
+        <v>172</v>
+      </c>
+      <c r="D8" t="n">
+        <v>54</v>
+      </c>
+      <c r="E8" t="n">
+        <v>118</v>
+      </c>
+      <c r="F8" t="n">
+        <v>41.7</v>
+      </c>
+      <c r="G8" t="n">
+        <v>57.4</v>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>Secretaría de Vivienda - Déficit Habitacional por barrios 2024 (SISBÉN). Corte único estructural.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>La Merced</t>
+        </is>
+      </c>
+      <c r="B9" t="n">
+        <v>54</v>
+      </c>
+      <c r="C9" t="n">
+        <v>26</v>
+      </c>
+      <c r="D9" t="n">
+        <v>1</v>
+      </c>
+      <c r="E9" t="n">
+        <v>25</v>
+      </c>
+      <c r="F9" t="n">
+        <v>48.1</v>
+      </c>
+      <c r="G9" t="n">
+        <v>57.4</v>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>Secretaría de Vivienda - Déficit Habitacional por barrios 2024 (SISBÉN). Corte único estructural.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>San Pascual</t>
+        </is>
+      </c>
+      <c r="B10" t="n">
+        <v>766</v>
+      </c>
+      <c r="C10" t="n">
+        <v>345</v>
+      </c>
+      <c r="D10" t="n">
+        <v>61</v>
+      </c>
+      <c r="E10" t="n">
+        <v>284</v>
+      </c>
+      <c r="F10" t="n">
+        <v>45</v>
+      </c>
+      <c r="G10" t="n">
+        <v>57.4</v>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>Secretaría de Vivienda - Déficit Habitacional por barrios 2024 (SISBÉN). Corte único estructural.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>El Calvario</t>
+        </is>
+      </c>
+      <c r="B11" t="n">
+        <v>113</v>
+      </c>
+      <c r="C11" t="n">
+        <v>52</v>
+      </c>
+      <c r="D11" t="n">
+        <v>9</v>
+      </c>
+      <c r="E11" t="n">
+        <v>43</v>
+      </c>
+      <c r="F11" t="n">
+        <v>46</v>
+      </c>
+      <c r="G11" t="n">
+        <v>57.4</v>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>Secretaría de Vivienda - Déficit Habitacional por barrios 2024 (SISBÉN). Corte único estructural.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>San Pedro</t>
+        </is>
+      </c>
+      <c r="B12" t="n">
+        <v>41</v>
+      </c>
+      <c r="C12" t="n">
+        <v>20</v>
+      </c>
+      <c r="D12" t="n">
+        <v>8</v>
+      </c>
+      <c r="E12" t="n">
+        <v>12</v>
+      </c>
+      <c r="F12" t="n">
+        <v>48.8</v>
+      </c>
+      <c r="G12" t="n">
+        <v>57.4</v>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>Secretaría de Vivienda - Déficit Habitacional por barrios 2024 (SISBÉN). Corte único estructural.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>San Nicolás</t>
+        </is>
+      </c>
+      <c r="B13" t="n">
+        <v>812</v>
+      </c>
+      <c r="C13" t="n">
+        <v>342</v>
+      </c>
+      <c r="D13" t="n">
+        <v>53</v>
+      </c>
+      <c r="E13" t="n">
+        <v>289</v>
+      </c>
+      <c r="F13" t="n">
+        <v>42.1</v>
+      </c>
+      <c r="G13" t="n">
+        <v>57.4</v>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>Secretaría de Vivienda - Déficit Habitacional por barrios 2024 (SISBÉN). Corte único estructural.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>El Hoyo</t>
+        </is>
+      </c>
+      <c r="B14" t="n">
+        <v>148</v>
+      </c>
+      <c r="C14" t="n">
+        <v>78</v>
+      </c>
+      <c r="D14" t="n">
+        <v>8</v>
+      </c>
+      <c r="E14" t="n">
+        <v>70</v>
+      </c>
+      <c r="F14" t="n">
+        <v>52.7</v>
+      </c>
+      <c r="G14" t="n">
+        <v>57.4</v>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>Secretaría de Vivienda - Déficit Habitacional por barrios 2024 (SISBÉN). Corte único estructural.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>El Piloto</t>
+        </is>
+      </c>
+      <c r="B15" t="n">
+        <v>211</v>
+      </c>
+      <c r="C15" t="n">
+        <v>103</v>
+      </c>
+      <c r="D15" t="n">
+        <v>17</v>
+      </c>
+      <c r="E15" t="n">
+        <v>86</v>
+      </c>
+      <c r="F15" t="n">
+        <v>48.8</v>
+      </c>
+      <c r="G15" t="n">
+        <v>57.4</v>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>Secretaría de Vivienda - Déficit Habitacional por barrios 2024 (SISBÉN). Corte único estructural.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>Navarro - La Chanca</t>
+        </is>
+      </c>
+      <c r="B16" t="n">
+        <v>154</v>
+      </c>
+      <c r="C16" t="n">
+        <v>64</v>
+      </c>
+      <c r="D16" t="n">
+        <v>6</v>
+      </c>
+      <c r="E16" t="n">
+        <v>58</v>
+      </c>
+      <c r="F16" t="n">
+        <v>41.6</v>
+      </c>
+      <c r="G16" t="n">
+        <v>57.4</v>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>Secretaría de Vivienda - Déficit Habitacional por barrios 2024 (SISBÉN). Corte único estructural.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>TOTAL Ciudad Paraíso (Comuna 3)</t>
+        </is>
+      </c>
+      <c r="B17" t="n">
+        <v>5912</v>
+      </c>
+      <c r="C17" t="n">
+        <v>2516</v>
+      </c>
+      <c r="D17" t="n">
+        <v>425</v>
+      </c>
+      <c r="E17" t="n">
+        <v>2091</v>
+      </c>
+      <c r="F17" t="n">
+        <v>42.6</v>
+      </c>
+      <c r="G17" t="n">
+        <v>57.4</v>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>Secretaría de Vivienda - Déficit Habitacional por barrios 2024 (SISBÉN). Corte único estructural.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:K5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -1569,7 +2254,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1837,7 +2522,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -2489,142 +3174,4 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:B10"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="34" customWidth="1" min="1" max="1"/>
-    <col width="40" customWidth="1" min="2" max="2"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>fuente</t>
-        </is>
-      </c>
-      <c r="B1" s="1" t="inlineStr">
-        <is>
-          <t>nota</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>Homicidios</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>Línea base por verificación espacial (Celda 4B); extensiones 2026 por spatial join al polígono.</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>Hurtos</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>Línea base por verificación espacial (Celda 4B); extensiones 2026 por spatial join al polígono.</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>Comparendos</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>Línea base por verificación espacial (Celda 4B); extensiones 2026 por spatial join al polígono.</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>VIF</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>Línea base por verificación espacial (Celda 4B); extensiones 2026 por spatial join al polígono.</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>Siniestros</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>Línea base por verificación espacial (Celda 4B); extensiones 2026 por spatial join al polígono.</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>Registro Mercantil (consolidado)</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>Línea base por verificación espacial (Celda 4B); extensiones 2026 por spatial join al polígono.</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>Censo Arboreo</t>
-        </is>
-      </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>Línea base por verificación espacial (Celda 4B); extensiones 2026 por spatial join al polígono.</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>Déficit Habitacional 2024</t>
-        </is>
-      </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>Línea base por verificación espacial (Celda 4B); extensiones 2026 por spatial join al polígono.</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>Educación SIMPADE</t>
-        </is>
-      </c>
-      <c r="B10" t="inlineStr">
-        <is>
-          <t>Línea base por verificación espacial (Celda 4B); extensiones 2026 por spatial join al polígono.</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
 </file>
</xml_diff>

<commit_message>
fix(nb08): vivienda filtrada a ZONA DE ESTUDIO (6 barrios del poligono: Guayaquil, San Juan Bosco, San Pascual, Santa Rosa, Sucre, El Calvario) via geojson recortado; habitabilidad 57.4->53.7 (deficit 46.3%); hoja Vivienda y EntornoU actualizados
</commit_message>
<xml_diff>
--- a/outputs/itt_ciudad_paraiso/ITT_Ciudad_Paraiso_Consolidado.xlsx
+++ b/outputs/itt_ciudad_paraiso/ITT_Ciudad_Paraiso_Consolidado.xlsx
@@ -509,13 +509,13 @@
         <v>65.06</v>
       </c>
       <c r="E2" t="n">
-        <v>53.36</v>
+        <v>52.13</v>
       </c>
       <c r="F2" t="n">
         <v>60.96</v>
       </c>
       <c r="G2" t="n">
-        <v>45.28</v>
+        <v>45.07</v>
       </c>
       <c r="H2" t="inlineStr">
         <is>
@@ -542,13 +542,13 @@
         <v>53.55</v>
       </c>
       <c r="E3" t="n">
-        <v>62.73</v>
+        <v>61.5</v>
       </c>
       <c r="F3" t="n">
         <v>64.98</v>
       </c>
       <c r="G3" t="n">
-        <v>54.14</v>
+        <v>53.93</v>
       </c>
       <c r="H3" t="inlineStr">
         <is>
@@ -575,13 +575,13 @@
         <v>33.2</v>
       </c>
       <c r="E4" t="n">
-        <v>62.6</v>
+        <v>61.37</v>
       </c>
       <c r="F4" t="n">
         <v>68.56</v>
       </c>
       <c r="G4" t="n">
-        <v>57.75</v>
+        <v>57.54</v>
       </c>
       <c r="H4" t="inlineStr">
         <is>
@@ -608,13 +608,13 @@
         <v>12.68</v>
       </c>
       <c r="E5" t="n">
-        <v>56.13</v>
+        <v>54.89</v>
       </c>
       <c r="F5" t="n">
         <v>67.3</v>
       </c>
       <c r="G5" t="n">
-        <v>66.62</v>
+        <v>66.41</v>
       </c>
       <c r="H5" t="inlineStr">
         <is>
@@ -1362,10 +1362,10 @@
         <v>66.7401</v>
       </c>
       <c r="F2" t="n">
-        <v>57.4</v>
+        <v>53.7</v>
       </c>
       <c r="G2" t="n">
-        <v>53.3643</v>
+        <v>52.1309</v>
       </c>
       <c r="H2" t="inlineStr">
         <is>
@@ -1395,10 +1395,10 @@
         <v>66.7401</v>
       </c>
       <c r="F3" t="n">
-        <v>57.4</v>
+        <v>53.7</v>
       </c>
       <c r="G3" t="n">
-        <v>62.7294</v>
+        <v>61.4961</v>
       </c>
       <c r="H3" t="inlineStr">
         <is>
@@ -1428,10 +1428,10 @@
         <v>66.7401</v>
       </c>
       <c r="F4" t="n">
-        <v>57.4</v>
+        <v>53.7</v>
       </c>
       <c r="G4" t="n">
-        <v>62.6017</v>
+        <v>61.3684</v>
       </c>
       <c r="H4" t="inlineStr">
         <is>
@@ -1461,10 +1461,10 @@
         <v>66.7401</v>
       </c>
       <c r="F5" t="n">
-        <v>57.4</v>
+        <v>53.7</v>
       </c>
       <c r="G5" t="n">
-        <v>56.1275</v>
+        <v>54.8942</v>
       </c>
       <c r="H5" t="inlineStr">
         <is>
@@ -1488,10 +1488,10 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H17"/>
+  <dimension ref="A1:H8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="33" customWidth="1" min="1" max="1"/>
+    <col width="35" customWidth="1" min="1" max="1"/>
     <col width="15" customWidth="1" min="2" max="2"/>
     <col width="22" customWidth="1" min="3" max="3"/>
     <col width="22" customWidth="1" min="4" max="4"/>
@@ -1546,480 +1546,210 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>El Nacional</t>
+          <t>Guayaquil</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>470</v>
+        <v>1028</v>
       </c>
       <c r="C2" t="n">
-        <v>198</v>
+        <v>477</v>
       </c>
       <c r="D2" t="n">
-        <v>17</v>
+        <v>42</v>
       </c>
       <c r="E2" t="n">
-        <v>181</v>
+        <v>435</v>
       </c>
       <c r="F2" t="n">
-        <v>42.1</v>
+        <v>46.4</v>
       </c>
       <c r="G2" t="n">
-        <v>57.4</v>
+        <v>53.7</v>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>Secretaría de Vivienda - Déficit Habitacional por barrios 2024 (SISBÉN). Corte único estructural.</t>
+          <t>Secretaría de Vivienda - Déficit Habitacional 2024 (SISBÉN), recortado al polígono de estudio. Corte único estructural.</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>El Peñón</t>
+          <t>San Juan Bosco</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>12</v>
+        <v>1120</v>
       </c>
       <c r="C3" t="n">
-        <v>6</v>
+        <v>558</v>
       </c>
       <c r="D3" t="n">
-        <v>0</v>
+        <v>158</v>
       </c>
       <c r="E3" t="n">
-        <v>6</v>
+        <v>400</v>
       </c>
       <c r="F3" t="n">
-        <v>50</v>
+        <v>49.8</v>
       </c>
       <c r="G3" t="n">
-        <v>57.4</v>
+        <v>53.7</v>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>Secretaría de Vivienda - Déficit Habitacional por barrios 2024 (SISBÉN). Corte único estructural.</t>
+          <t>Secretaría de Vivienda - Déficit Habitacional 2024 (SISBÉN), recortado al polígono de estudio. Corte único estructural.</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>San Antonio</t>
+          <t>San Pascual</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>216</v>
+        <v>766</v>
       </c>
       <c r="C4" t="n">
-        <v>94</v>
+        <v>345</v>
       </c>
       <c r="D4" t="n">
-        <v>6</v>
+        <v>61</v>
       </c>
       <c r="E4" t="n">
-        <v>88</v>
+        <v>284</v>
       </c>
       <c r="F4" t="n">
-        <v>43.5</v>
+        <v>45</v>
       </c>
       <c r="G4" t="n">
-        <v>57.4</v>
+        <v>53.7</v>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>Secretaría de Vivienda - Déficit Habitacional por barrios 2024 (SISBÉN). Corte único estructural.</t>
+          <t>Secretaría de Vivienda - Déficit Habitacional 2024 (SISBÉN), recortado al polígono de estudio. Corte único estructural.</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>San Cayetano</t>
+          <t>Santa Rosa</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>754</v>
+        <v>412</v>
       </c>
       <c r="C5" t="n">
-        <v>240</v>
+        <v>172</v>
       </c>
       <c r="D5" t="n">
-        <v>12</v>
+        <v>54</v>
       </c>
       <c r="E5" t="n">
-        <v>228</v>
+        <v>118</v>
       </c>
       <c r="F5" t="n">
-        <v>31.8</v>
+        <v>41.7</v>
       </c>
       <c r="G5" t="n">
-        <v>57.4</v>
+        <v>53.7</v>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>Secretaría de Vivienda - Déficit Habitacional por barrios 2024 (SISBÉN). Corte único estructural.</t>
+          <t>Secretaría de Vivienda - Déficit Habitacional 2024 (SISBÉN), recortado al polígono de estudio. Corte único estructural.</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Los Libertadores</t>
+          <t>Sucre</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>629</v>
+        <v>2363</v>
       </c>
       <c r="C6" t="n">
-        <v>218</v>
+        <v>1082</v>
       </c>
       <c r="D6" t="n">
-        <v>15</v>
+        <v>223</v>
       </c>
       <c r="E6" t="n">
-        <v>203</v>
+        <v>859</v>
       </c>
       <c r="F6" t="n">
-        <v>34.7</v>
+        <v>45.8</v>
       </c>
       <c r="G6" t="n">
-        <v>57.4</v>
+        <v>53.7</v>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>Secretaría de Vivienda - Déficit Habitacional por barrios 2024 (SISBÉN). Corte único estructural.</t>
+          <t>Secretaría de Vivienda - Déficit Habitacional 2024 (SISBÉN), recortado al polígono de estudio. Corte único estructural.</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>San Juan Bosco</t>
+          <t>El Calvario</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>1120</v>
+        <v>113</v>
       </c>
       <c r="C7" t="n">
-        <v>558</v>
+        <v>52</v>
       </c>
       <c r="D7" t="n">
-        <v>158</v>
+        <v>9</v>
       </c>
       <c r="E7" t="n">
-        <v>400</v>
+        <v>43</v>
       </c>
       <c r="F7" t="n">
-        <v>49.8</v>
+        <v>46</v>
       </c>
       <c r="G7" t="n">
-        <v>57.4</v>
+        <v>53.7</v>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>Secretaría de Vivienda - Déficit Habitacional por barrios 2024 (SISBÉN). Corte único estructural.</t>
+          <t>Secretaría de Vivienda - Déficit Habitacional 2024 (SISBÉN), recortado al polígono de estudio. Corte único estructural.</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Santa Rosa</t>
+          <t>TOTAL zona estudio Ciudad Paraíso</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>412</v>
+        <v>5802</v>
       </c>
       <c r="C8" t="n">
-        <v>172</v>
+        <v>2686</v>
       </c>
       <c r="D8" t="n">
-        <v>54</v>
+        <v>547</v>
       </c>
       <c r="E8" t="n">
-        <v>118</v>
+        <v>2139</v>
       </c>
       <c r="F8" t="n">
-        <v>41.7</v>
+        <v>46.3</v>
       </c>
       <c r="G8" t="n">
-        <v>57.4</v>
+        <v>53.7</v>
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>Secretaría de Vivienda - Déficit Habitacional por barrios 2024 (SISBÉN). Corte único estructural.</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>La Merced</t>
-        </is>
-      </c>
-      <c r="B9" t="n">
-        <v>54</v>
-      </c>
-      <c r="C9" t="n">
-        <v>26</v>
-      </c>
-      <c r="D9" t="n">
-        <v>1</v>
-      </c>
-      <c r="E9" t="n">
-        <v>25</v>
-      </c>
-      <c r="F9" t="n">
-        <v>48.1</v>
-      </c>
-      <c r="G9" t="n">
-        <v>57.4</v>
-      </c>
-      <c r="H9" t="inlineStr">
-        <is>
-          <t>Secretaría de Vivienda - Déficit Habitacional por barrios 2024 (SISBÉN). Corte único estructural.</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>San Pascual</t>
-        </is>
-      </c>
-      <c r="B10" t="n">
-        <v>766</v>
-      </c>
-      <c r="C10" t="n">
-        <v>345</v>
-      </c>
-      <c r="D10" t="n">
-        <v>61</v>
-      </c>
-      <c r="E10" t="n">
-        <v>284</v>
-      </c>
-      <c r="F10" t="n">
-        <v>45</v>
-      </c>
-      <c r="G10" t="n">
-        <v>57.4</v>
-      </c>
-      <c r="H10" t="inlineStr">
-        <is>
-          <t>Secretaría de Vivienda - Déficit Habitacional por barrios 2024 (SISBÉN). Corte único estructural.</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>El Calvario</t>
-        </is>
-      </c>
-      <c r="B11" t="n">
-        <v>113</v>
-      </c>
-      <c r="C11" t="n">
-        <v>52</v>
-      </c>
-      <c r="D11" t="n">
-        <v>9</v>
-      </c>
-      <c r="E11" t="n">
-        <v>43</v>
-      </c>
-      <c r="F11" t="n">
-        <v>46</v>
-      </c>
-      <c r="G11" t="n">
-        <v>57.4</v>
-      </c>
-      <c r="H11" t="inlineStr">
-        <is>
-          <t>Secretaría de Vivienda - Déficit Habitacional por barrios 2024 (SISBÉN). Corte único estructural.</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="inlineStr">
-        <is>
-          <t>San Pedro</t>
-        </is>
-      </c>
-      <c r="B12" t="n">
-        <v>41</v>
-      </c>
-      <c r="C12" t="n">
-        <v>20</v>
-      </c>
-      <c r="D12" t="n">
-        <v>8</v>
-      </c>
-      <c r="E12" t="n">
-        <v>12</v>
-      </c>
-      <c r="F12" t="n">
-        <v>48.8</v>
-      </c>
-      <c r="G12" t="n">
-        <v>57.4</v>
-      </c>
-      <c r="H12" t="inlineStr">
-        <is>
-          <t>Secretaría de Vivienda - Déficit Habitacional por barrios 2024 (SISBÉN). Corte único estructural.</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="inlineStr">
-        <is>
-          <t>San Nicolás</t>
-        </is>
-      </c>
-      <c r="B13" t="n">
-        <v>812</v>
-      </c>
-      <c r="C13" t="n">
-        <v>342</v>
-      </c>
-      <c r="D13" t="n">
-        <v>53</v>
-      </c>
-      <c r="E13" t="n">
-        <v>289</v>
-      </c>
-      <c r="F13" t="n">
-        <v>42.1</v>
-      </c>
-      <c r="G13" t="n">
-        <v>57.4</v>
-      </c>
-      <c r="H13" t="inlineStr">
-        <is>
-          <t>Secretaría de Vivienda - Déficit Habitacional por barrios 2024 (SISBÉN). Corte único estructural.</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" t="inlineStr">
-        <is>
-          <t>El Hoyo</t>
-        </is>
-      </c>
-      <c r="B14" t="n">
-        <v>148</v>
-      </c>
-      <c r="C14" t="n">
-        <v>78</v>
-      </c>
-      <c r="D14" t="n">
-        <v>8</v>
-      </c>
-      <c r="E14" t="n">
-        <v>70</v>
-      </c>
-      <c r="F14" t="n">
-        <v>52.7</v>
-      </c>
-      <c r="G14" t="n">
-        <v>57.4</v>
-      </c>
-      <c r="H14" t="inlineStr">
-        <is>
-          <t>Secretaría de Vivienda - Déficit Habitacional por barrios 2024 (SISBÉN). Corte único estructural.</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" t="inlineStr">
-        <is>
-          <t>El Piloto</t>
-        </is>
-      </c>
-      <c r="B15" t="n">
-        <v>211</v>
-      </c>
-      <c r="C15" t="n">
-        <v>103</v>
-      </c>
-      <c r="D15" t="n">
-        <v>17</v>
-      </c>
-      <c r="E15" t="n">
-        <v>86</v>
-      </c>
-      <c r="F15" t="n">
-        <v>48.8</v>
-      </c>
-      <c r="G15" t="n">
-        <v>57.4</v>
-      </c>
-      <c r="H15" t="inlineStr">
-        <is>
-          <t>Secretaría de Vivienda - Déficit Habitacional por barrios 2024 (SISBÉN). Corte único estructural.</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" t="inlineStr">
-        <is>
-          <t>Navarro - La Chanca</t>
-        </is>
-      </c>
-      <c r="B16" t="n">
-        <v>154</v>
-      </c>
-      <c r="C16" t="n">
-        <v>64</v>
-      </c>
-      <c r="D16" t="n">
-        <v>6</v>
-      </c>
-      <c r="E16" t="n">
-        <v>58</v>
-      </c>
-      <c r="F16" t="n">
-        <v>41.6</v>
-      </c>
-      <c r="G16" t="n">
-        <v>57.4</v>
-      </c>
-      <c r="H16" t="inlineStr">
-        <is>
-          <t>Secretaría de Vivienda - Déficit Habitacional por barrios 2024 (SISBÉN). Corte único estructural.</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" t="inlineStr">
-        <is>
-          <t>TOTAL Ciudad Paraíso (Comuna 3)</t>
-        </is>
-      </c>
-      <c r="B17" t="n">
-        <v>5912</v>
-      </c>
-      <c r="C17" t="n">
-        <v>2516</v>
-      </c>
-      <c r="D17" t="n">
-        <v>425</v>
-      </c>
-      <c r="E17" t="n">
-        <v>2091</v>
-      </c>
-      <c r="F17" t="n">
-        <v>42.6</v>
-      </c>
-      <c r="G17" t="n">
-        <v>57.4</v>
-      </c>
-      <c r="H17" t="inlineStr">
-        <is>
-          <t>Secretaría de Vivienda - Déficit Habitacional por barrios 2024 (SISBÉN). Corte único estructural.</t>
+          <t>Secretaría de Vivienda - Déficit Habitacional 2024 (SISBÉN), recortado al polígono de estudio. Corte único estructural.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat(nb08): vivienda por SPATIAL JOIN + PRORRATEO de area con shapefile SISBEN (386 barrios Cali); habitabilidad 53.9 (1158 hogares prorrateados, deficit 46.1%); subsidios=0 en zona documentado; hoja Vivienda con detalle espacial
</commit_message>
<xml_diff>
--- a/outputs/itt_ciudad_paraiso/ITT_Ciudad_Paraiso_Consolidado.xlsx
+++ b/outputs/itt_ciudad_paraiso/ITT_Ciudad_Paraiso_Consolidado.xlsx
@@ -509,13 +509,13 @@
         <v>65.06</v>
       </c>
       <c r="E2" t="n">
-        <v>52.13</v>
+        <v>52.2</v>
       </c>
       <c r="F2" t="n">
         <v>60.96</v>
       </c>
       <c r="G2" t="n">
-        <v>45.07</v>
+        <v>45.08</v>
       </c>
       <c r="H2" t="inlineStr">
         <is>
@@ -542,13 +542,13 @@
         <v>53.55</v>
       </c>
       <c r="E3" t="n">
-        <v>61.5</v>
+        <v>61.56</v>
       </c>
       <c r="F3" t="n">
         <v>64.98</v>
       </c>
       <c r="G3" t="n">
-        <v>53.93</v>
+        <v>53.94</v>
       </c>
       <c r="H3" t="inlineStr">
         <is>
@@ -575,13 +575,13 @@
         <v>33.2</v>
       </c>
       <c r="E4" t="n">
-        <v>61.37</v>
+        <v>61.44</v>
       </c>
       <c r="F4" t="n">
         <v>68.56</v>
       </c>
       <c r="G4" t="n">
-        <v>57.54</v>
+        <v>57.55</v>
       </c>
       <c r="H4" t="inlineStr">
         <is>
@@ -608,13 +608,13 @@
         <v>12.68</v>
       </c>
       <c r="E5" t="n">
-        <v>54.89</v>
+        <v>54.96</v>
       </c>
       <c r="F5" t="n">
         <v>67.3</v>
       </c>
       <c r="G5" t="n">
-        <v>66.41</v>
+        <v>66.42</v>
       </c>
       <c r="H5" t="inlineStr">
         <is>
@@ -1362,10 +1362,10 @@
         <v>66.7401</v>
       </c>
       <c r="F2" t="n">
-        <v>53.7</v>
+        <v>53.9</v>
       </c>
       <c r="G2" t="n">
-        <v>52.1309</v>
+        <v>52.1976</v>
       </c>
       <c r="H2" t="inlineStr">
         <is>
@@ -1395,10 +1395,10 @@
         <v>66.7401</v>
       </c>
       <c r="F3" t="n">
-        <v>53.7</v>
+        <v>53.9</v>
       </c>
       <c r="G3" t="n">
-        <v>61.4961</v>
+        <v>61.5628</v>
       </c>
       <c r="H3" t="inlineStr">
         <is>
@@ -1428,10 +1428,10 @@
         <v>66.7401</v>
       </c>
       <c r="F4" t="n">
-        <v>53.7</v>
+        <v>53.9</v>
       </c>
       <c r="G4" t="n">
-        <v>61.3684</v>
+        <v>61.435</v>
       </c>
       <c r="H4" t="inlineStr">
         <is>
@@ -1461,10 +1461,10 @@
         <v>66.7401</v>
       </c>
       <c r="F5" t="n">
-        <v>53.7</v>
+        <v>53.9</v>
       </c>
       <c r="G5" t="n">
-        <v>54.8942</v>
+        <v>54.9608</v>
       </c>
       <c r="H5" t="inlineStr">
         <is>
@@ -1488,17 +1488,22 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H8"/>
+  <dimension ref="A1:M7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="35" customWidth="1" min="1" max="1"/>
-    <col width="15" customWidth="1" min="2" max="2"/>
+    <col width="34" customWidth="1" min="1" max="1"/>
+    <col width="22" customWidth="1" min="2" max="2"/>
     <col width="22" customWidth="1" min="3" max="3"/>
-    <col width="22" customWidth="1" min="4" max="4"/>
-    <col width="21" customWidth="1" min="5" max="5"/>
-    <col width="16" customWidth="1" min="6" max="6"/>
-    <col width="21" customWidth="1" min="7" max="7"/>
-    <col width="40" customWidth="1" min="8" max="8"/>
+    <col width="29" customWidth="1" min="4" max="4"/>
+    <col width="28" customWidth="1" min="5" max="5"/>
+    <col width="17" customWidth="1" min="6" max="6"/>
+    <col width="17" customWidth="1" min="7" max="7"/>
+    <col width="17" customWidth="1" min="8" max="8"/>
+    <col width="16" customWidth="1" min="9" max="9"/>
+    <col width="21" customWidth="1" min="10" max="10"/>
+    <col width="40" customWidth="1" min="11" max="11"/>
+    <col width="32" customWidth="1" min="12" max="12"/>
+    <col width="40" customWidth="1" min="13" max="13"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1509,67 +1514,109 @@
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>total_hogares</t>
+          <t>hogares_barrio_total</t>
         </is>
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>deficit_habitacional</t>
+          <t>deficit_barrio_total</t>
         </is>
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>deficit_cuantitativo</t>
+          <t>deficit_cuantitativo_barrio</t>
         </is>
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
-          <t>deficit_cualitativo</t>
+          <t>deficit_cualitativo_barrio</t>
         </is>
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
+          <t>pct_area_dentro</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>hogares_en_zona</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>deficit_en_zona</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
           <t>tasa_deficit_%</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>habitabilidad_score</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>fuente</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>subsidios_mejoramiento_en_zona</t>
+        </is>
+      </c>
+      <c r="M1" s="1" t="inlineStr">
+        <is>
+          <t>nota_subsidios</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Guayaquil</t>
+          <t>San Pascual</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>1028</v>
+        <v>766</v>
       </c>
       <c r="C2" t="n">
-        <v>477</v>
+        <v>345</v>
       </c>
       <c r="D2" t="n">
-        <v>42</v>
+        <v>61</v>
       </c>
       <c r="E2" t="n">
-        <v>435</v>
+        <v>284</v>
       </c>
       <c r="F2" t="n">
-        <v>46.4</v>
+        <v>98.09999999999999</v>
       </c>
       <c r="G2" t="n">
-        <v>53.7</v>
-      </c>
-      <c r="H2" t="inlineStr">
-        <is>
-          <t>Secretaría de Vivienda - Déficit Habitacional 2024 (SISBÉN), recortado al polígono de estudio. Corte único estructural.</t>
+        <v>751</v>
+      </c>
+      <c r="H2" t="n">
+        <v>338</v>
+      </c>
+      <c r="I2" t="n">
+        <v>45</v>
+      </c>
+      <c r="J2" t="n">
+        <v>53.9</v>
+      </c>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>Secretaría de Vivienda - Déficit Habitacional SISBÉN 2024. Spatial join + prorrateo por área al polígono de estudio. Corte único estructural.</t>
+        </is>
+      </c>
+      <c r="L2" t="n">
+        <v>0</v>
+      </c>
+      <c r="M2" t="inlineStr">
+        <is>
+          <t>Subsidios de mejoramiento de vivienda 2024-2026: 0 en la zona de estudio (programa dirigido a comunas de ladera/periferia, no al centro).</t>
         </is>
       </c>
     </row>
@@ -1592,44 +1639,78 @@
         <v>400</v>
       </c>
       <c r="F3" t="n">
+        <v>25.9</v>
+      </c>
+      <c r="G3" t="n">
+        <v>290</v>
+      </c>
+      <c r="H3" t="n">
+        <v>144</v>
+      </c>
+      <c r="I3" t="n">
         <v>49.8</v>
       </c>
-      <c r="G3" t="n">
-        <v>53.7</v>
-      </c>
-      <c r="H3" t="inlineStr">
-        <is>
-          <t>Secretaría de Vivienda - Déficit Habitacional 2024 (SISBÉN), recortado al polígono de estudio. Corte único estructural.</t>
+      <c r="J3" t="n">
+        <v>53.9</v>
+      </c>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>Secretaría de Vivienda - Déficit Habitacional SISBÉN 2024. Spatial join + prorrateo por área al polígono de estudio. Corte único estructural.</t>
+        </is>
+      </c>
+      <c r="L3" t="n">
+        <v>0</v>
+      </c>
+      <c r="M3" t="inlineStr">
+        <is>
+          <t>Subsidios de mejoramiento de vivienda 2024-2026: 0 en la zona de estudio (programa dirigido a comunas de ladera/periferia, no al centro).</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>San Pascual</t>
+          <t>El Calvario</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>766</v>
+        <v>113</v>
       </c>
       <c r="C4" t="n">
-        <v>345</v>
+        <v>52</v>
       </c>
       <c r="D4" t="n">
-        <v>61</v>
+        <v>9</v>
       </c>
       <c r="E4" t="n">
-        <v>284</v>
+        <v>43</v>
       </c>
       <c r="F4" t="n">
-        <v>45</v>
+        <v>51.9</v>
       </c>
       <c r="G4" t="n">
-        <v>53.7</v>
-      </c>
-      <c r="H4" t="inlineStr">
-        <is>
-          <t>Secretaría de Vivienda - Déficit Habitacional 2024 (SISBÉN), recortado al polígono de estudio. Corte único estructural.</t>
+        <v>59</v>
+      </c>
+      <c r="H4" t="n">
+        <v>27</v>
+      </c>
+      <c r="I4" t="n">
+        <v>46</v>
+      </c>
+      <c r="J4" t="n">
+        <v>53.9</v>
+      </c>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>Secretaría de Vivienda - Déficit Habitacional SISBÉN 2024. Spatial join + prorrateo por área al polígono de estudio. Corte único estructural.</t>
+        </is>
+      </c>
+      <c r="L4" t="n">
+        <v>0</v>
+      </c>
+      <c r="M4" t="inlineStr">
+        <is>
+          <t>Subsidios de mejoramiento de vivienda 2024-2026: 0 en la zona de estudio (programa dirigido a comunas de ladera/periferia, no al centro).</t>
         </is>
       </c>
     </row>
@@ -1652,14 +1733,31 @@
         <v>118</v>
       </c>
       <c r="F5" t="n">
+        <v>13.8</v>
+      </c>
+      <c r="G5" t="n">
+        <v>57</v>
+      </c>
+      <c r="H5" t="n">
+        <v>24</v>
+      </c>
+      <c r="I5" t="n">
         <v>41.7</v>
       </c>
-      <c r="G5" t="n">
-        <v>53.7</v>
-      </c>
-      <c r="H5" t="inlineStr">
-        <is>
-          <t>Secretaría de Vivienda - Déficit Habitacional 2024 (SISBÉN), recortado al polígono de estudio. Corte único estructural.</t>
+      <c r="J5" t="n">
+        <v>53.9</v>
+      </c>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>Secretaría de Vivienda - Déficit Habitacional SISBÉN 2024. Spatial join + prorrateo por área al polígono de estudio. Corte único estructural.</t>
+        </is>
+      </c>
+      <c r="L5" t="n">
+        <v>0</v>
+      </c>
+      <c r="M5" t="inlineStr">
+        <is>
+          <t>Subsidios de mejoramiento de vivienda 2024-2026: 0 en la zona de estudio (programa dirigido a comunas de ladera/periferia, no al centro).</t>
         </is>
       </c>
     </row>
@@ -1682,74 +1780,68 @@
         <v>859</v>
       </c>
       <c r="F6" t="n">
+        <v>0</v>
+      </c>
+      <c r="G6" t="n">
+        <v>1</v>
+      </c>
+      <c r="H6" t="n">
+        <v>1</v>
+      </c>
+      <c r="I6" t="n">
         <v>45.8</v>
       </c>
-      <c r="G6" t="n">
-        <v>53.7</v>
-      </c>
-      <c r="H6" t="inlineStr">
-        <is>
-          <t>Secretaría de Vivienda - Déficit Habitacional 2024 (SISBÉN), recortado al polígono de estudio. Corte único estructural.</t>
+      <c r="J6" t="n">
+        <v>53.9</v>
+      </c>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>Secretaría de Vivienda - Déficit Habitacional SISBÉN 2024. Spatial join + prorrateo por área al polígono de estudio. Corte único estructural.</t>
+        </is>
+      </c>
+      <c r="L6" t="n">
+        <v>0</v>
+      </c>
+      <c r="M6" t="inlineStr">
+        <is>
+          <t>Subsidios de mejoramiento de vivienda 2024-2026: 0 en la zona de estudio (programa dirigido a comunas de ladera/periferia, no al centro).</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>El Calvario</t>
-        </is>
-      </c>
-      <c r="B7" t="n">
-        <v>113</v>
-      </c>
-      <c r="C7" t="n">
-        <v>52</v>
-      </c>
-      <c r="D7" t="n">
-        <v>9</v>
-      </c>
-      <c r="E7" t="n">
-        <v>43</v>
-      </c>
-      <c r="F7" t="n">
-        <v>46</v>
-      </c>
+          <t>TOTAL zona estudio (prorrateado)</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr"/>
+      <c r="C7" t="inlineStr"/>
+      <c r="D7" t="inlineStr"/>
+      <c r="E7" t="inlineStr"/>
+      <c r="F7" t="inlineStr"/>
       <c r="G7" t="n">
-        <v>53.7</v>
-      </c>
-      <c r="H7" t="inlineStr">
-        <is>
-          <t>Secretaría de Vivienda - Déficit Habitacional 2024 (SISBÉN), recortado al polígono de estudio. Corte único estructural.</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>TOTAL zona estudio Ciudad Paraíso</t>
-        </is>
-      </c>
-      <c r="B8" t="n">
-        <v>5802</v>
-      </c>
-      <c r="C8" t="n">
-        <v>2686</v>
-      </c>
-      <c r="D8" t="n">
-        <v>547</v>
-      </c>
-      <c r="E8" t="n">
-        <v>2139</v>
-      </c>
-      <c r="F8" t="n">
-        <v>46.3</v>
-      </c>
-      <c r="G8" t="n">
-        <v>53.7</v>
-      </c>
-      <c r="H8" t="inlineStr">
-        <is>
-          <t>Secretaría de Vivienda - Déficit Habitacional 2024 (SISBÉN), recortado al polígono de estudio. Corte único estructural.</t>
+        <v>1158</v>
+      </c>
+      <c r="H7" t="n">
+        <v>534</v>
+      </c>
+      <c r="I7" t="n">
+        <v>46.1</v>
+      </c>
+      <c r="J7" t="n">
+        <v>53.9</v>
+      </c>
+      <c r="K7" t="inlineStr">
+        <is>
+          <t>Secretaría de Vivienda - Déficit Habitacional SISBÉN 2024. Spatial join + prorrateo por área al polígono de estudio. Corte único estructural.</t>
+        </is>
+      </c>
+      <c r="L7" t="n">
+        <v>0</v>
+      </c>
+      <c r="M7" t="inlineStr">
+        <is>
+          <t>Subsidios de mejoramiento de vivienda 2024-2026: 0 en la zona de estudio (programa dirigido a comunas de ladera/periferia, no al centro).</t>
         </is>
       </c>
     </row>

</xml_diff>